<commit_message>
Actualizar a ControlPro V10 Architecture Lock
</commit_message>
<xml_diff>
--- a/deliverables/SAMPLE_BOM_PRICEGUARD.xlsx
+++ b/deliverables/SAMPLE_BOM_PRICEGUARD.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ControlPro Advisor OS V9 - BOM cotizable</t>
+          <t>ControlPro Advisor OS V10 - BOM cotizable</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Contactor subir</t>
+          <t>Contactor de línea / seguridad para VFD</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -828,7 +828,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>contactor_rev</t>
+          <t>vfd</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Contactor bajar</t>
+          <t>Variador de frecuencia</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -851,33 +851,33 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Cuenca Control Supply</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>LC1D32G7</t>
+          <t>ACS580-01-039A-4</t>
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>82</v>
+        <v>1180</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>82</v>
+        <v>1180</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>referencial fuerte</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media-alta</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="N8" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
@@ -900,24 +900,24 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (91.4%). Schneider LC1D32G7, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (80.7%). ABB ACS580-01-039A-4, Cuenca Control Supply, Cuenca.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>mechanical_interlock</t>
+          <t>line_reactor</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Fuerza</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Enclavamiento mecánico</t>
+          <t>Reactor de línea</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -930,46 +930,46 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Suministros El Oro</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>Genérico industrial</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>LAD9R1V</t>
+          <t>LR-25HP-460</t>
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>27</v>
+        <v>168</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>27</v>
+        <v>168</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>referencial</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>verde</t>
+          <t>amarillo</t>
         </is>
       </c>
       <c r="N9" s="3" t="n">
-        <v>88.2</v>
+        <v>75</v>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
+          <t>Usar como referencia; enviar RFQ si el proyecto es sensible a precio o plazo.</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
@@ -979,24 +979,24 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (88.2%). Schneider LAD9R1V, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: AMARILLO (75.0%). Genérico industrial LR-25HP-460, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>phase_monitor</t>
+          <t>braking_resistor</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Fuerza</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Relé monitor de fase</t>
+          <t>Resistencia de frenado</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -1009,73 +1009,73 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Automatización Andina</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>Danfoss</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>RM22TR33</t>
+          <t>BR-25HP</t>
         </is>
       </c>
       <c r="I10" s="4" t="n">
-        <v>94</v>
+        <v>247.5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>94</v>
+        <v>247.5</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>estimado corregido</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>baja</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>verde</t>
+          <t>rojo</t>
         </is>
       </c>
       <c r="N10" s="3" t="n">
-        <v>86.3</v>
+        <v>50.8</v>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
+          <t>Precio fuera de confianza. Usar mediana temporal y enviar RFQ a varios proveedores.</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>available</t>
+          <t>quote_needed</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.3%). Schneider RM22TR33, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: ROJO (50.8%). Danfoss BR-25HP, Automatización Andina, Quito. Alertas: stock no confirmado. Se aplicó autocorrección por banda de mercado.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>control_transformer</t>
+          <t>phase_monitor</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Transformador de control</t>
+          <t>Relé monitor de fase</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -1088,24 +1088,24 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Suministros El Oro</t>
+          <t>ElectroIndustrial Guayaquil</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Genérico industrial</t>
+          <t>Schneider</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>TC-2KVA</t>
+          <t>RM22TR33</t>
         </is>
       </c>
       <c r="I11" s="4" t="n">
-        <v>125</v>
+        <v>94</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>125</v>
+        <v>94</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
         </is>
       </c>
       <c r="N11" s="3" t="n">
-        <v>86.2</v>
+        <v>86.3</v>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
@@ -1137,24 +1137,24 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.2%). Genérico industrial TC-2KVA, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (86.3%). Schneider RM22TR33, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>cabinet</t>
+          <t>control_transformer</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Tablero</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Gabinete industrial</t>
+          <t>Transformador de control</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -1172,19 +1172,19 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Metálico Nacional</t>
+          <t>Genérico industrial</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>MN-604025</t>
+          <t>TC-2KVA</t>
         </is>
       </c>
       <c r="I12" s="4" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="N12" s="3" t="n">
-        <v>84.90000000000001</v>
+        <v>86.2</v>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
@@ -1216,24 +1216,24 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (84.9%). Metálico Nacional MN-604025, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (86.2%). Genérico industrial TC-2KVA, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>estop</t>
+          <t>cabinet</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Tablero</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Paro de emergencia</t>
+          <t>Gabinete industrial</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -1246,24 +1246,24 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Suministros El Oro</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>Metálico Nacional</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>XB4BS542</t>
+          <t>MN-604025</t>
         </is>
       </c>
       <c r="I13" s="4" t="n">
-        <v>24</v>
+        <v>135</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>24</v>
+        <v>135</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="N13" s="3" t="n">
-        <v>87.2</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
@@ -1295,24 +1295,24 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (87.2%). Schneider XB4BS542, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (84.9%). Metálico Nacional MN-604025, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>pushbuttons</t>
+          <t>estop</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Botonera de mando</t>
+          <t>Paro de emergencia</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -1335,14 +1335,14 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>XB4 Kit</t>
+          <t>XB4BS542</t>
         </is>
       </c>
       <c r="I14" s="4" t="n">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="N14" s="3" t="n">
-        <v>86.5</v>
+        <v>87.2</v>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
@@ -1374,28 +1374,28 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.5%). Schneider XB4 Kit, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (87.2%). Schneider XB4BS542, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>limit_switches</t>
+          <t>pushbuttons</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Finales de carrera</t>
+          <t>Botonera de mando</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
@@ -1414,14 +1414,14 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>XCK-M</t>
+          <t>XB4 Kit</t>
         </is>
       </c>
       <c r="I15" s="4" t="n">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="N15" s="3" t="n">
-        <v>86.8</v>
+        <v>86.5</v>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
@@ -1453,28 +1453,28 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.8%). Schneider XCK-M, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (86.5%). Schneider XB4 Kit, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>brake_rectifier</t>
+          <t>limit_switches</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Control/rectificador de freno</t>
+          <t>Finales de carrera</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
@@ -1483,33 +1483,33 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Proveedor Premium Quito</t>
+          <t>ElectroIndustrial Guayaquil</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Bonfiglioli</t>
+          <t>Schneider</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>BRE120</t>
+          <t>XCK-M</t>
         </is>
       </c>
       <c r="I16" s="4" t="n">
-        <v>142</v>
+        <v>38</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>142</v>
+        <v>76</v>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>referencial</t>
+          <t>confirmado</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="N16" s="3" t="n">
-        <v>77.7</v>
+        <v>86.8</v>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
@@ -1532,24 +1532,24 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (77.7%). Bonfiglioli BRE120, Proveedor Premium Quito, Quito.</t>
+          <t>PriceGuard: VERDE (86.8%). Schneider XCK-M, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>vfd</t>
+          <t>brake_rectifier</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Fuerza</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Variador de frecuencia</t>
+          <t>Control/rectificador de freno</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -1562,33 +1562,33 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Cuenca Control Supply</t>
+          <t>Proveedor Premium Quito</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Bonfiglioli</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>ACS580-01-039A-4</t>
+          <t>BRE120</t>
         </is>
       </c>
       <c r="I17" s="4" t="n">
-        <v>1180</v>
+        <v>142</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>1180</v>
+        <v>142</v>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>referencial fuerte</t>
+          <t>referencial</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>media-alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="N17" s="3" t="n">
-        <v>80.7</v>
+        <v>77.7</v>
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
@@ -1611,24 +1611,24 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (80.7%). ABB ACS580-01-039A-4, Cuenca Control Supply, Cuenca.</t>
+          <t>PriceGuard: VERDE (77.7%). Bonfiglioli BRE120, Proveedor Premium Quito, Quito.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>line_reactor</t>
+          <t>label_package</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Fuerza</t>
+          <t>Taller</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Reactor de línea</t>
+          <t>Etiquetado premium</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -1646,41 +1646,41 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Genérico industrial</t>
+          <t>Genérico</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>LR-25HP-460</t>
+          <t>LABEL-KIT</t>
         </is>
       </c>
       <c r="I18" s="4" t="n">
-        <v>168</v>
+        <v>32</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>168</v>
+        <v>32</v>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>referencial</t>
+          <t>confirmado</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>amarillo</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="N18" s="3" t="n">
-        <v>75</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>Usar como referencia; enviar RFQ si el proyecto es sensible a precio o plazo.</t>
+          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
         </is>
       </c>
       <c r="P18" s="3" t="inlineStr">
@@ -1690,24 +1690,24 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: AMARILLO (75.0%). Genérico industrial LR-25HP-460, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (81.1%). Genérico LABEL-KIT, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>braking_resistor</t>
+          <t>terminal_blocks</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Fuerza</t>
+          <t>Cableado</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Resistencia de frenado</t>
+          <t>Borneras, puentes y marcadores</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -1720,73 +1720,73 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Automatización Andina</t>
+          <t>Suministros El Oro</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Danfoss</t>
+          <t>Genérico</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>BR-25HP</t>
+          <t>TB-KIT-30</t>
         </is>
       </c>
       <c r="I19" s="4" t="n">
-        <v>247.5</v>
+        <v>38</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>247.5</v>
+        <v>38</v>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>estimado corregido</t>
+          <t>confirmado</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>rojo</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="N19" s="3" t="n">
-        <v>50.8</v>
+        <v>86.5</v>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Precio fuera de confianza. Usar mediana temporal y enviar RFQ a varios proveedores.</t>
+          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
         </is>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>quote_needed</t>
+          <t>available</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: ROJO (50.8%). Danfoss BR-25HP, Automatización Andina, Quito. Alertas: stock no confirmado. Se aplicó autocorrección por banda de mercado.</t>
+          <t>PriceGuard: VERDE (86.5%). Genérico TB-KIT-30, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>label_package</t>
+          <t>wiring_pack</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Taller</t>
+          <t>Cableado</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Etiquetado premium</t>
+          <t>Consumibles de cableado de tablero</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -1809,14 +1809,14 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>LABEL-KIT</t>
+          <t>WP-LOCAL</t>
         </is>
       </c>
       <c r="I20" s="4" t="n">
-        <v>32</v>
+        <v>98</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>32</v>
+        <v>98</v>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="N20" s="3" t="n">
-        <v>81.09999999999999</v>
+        <v>85.8</v>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
@@ -1848,14 +1848,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (81.1%). Genérico LABEL-KIT, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (85.8%). Genérico WP-LOCAL, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>terminal_blocks</t>
+          <t>power_cable</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1865,15 +1865,15 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Borneras, puentes y marcadores</t>
+          <t>Conductor de fuerza</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>1</v>
+        <v>53.1</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1883,19 +1883,19 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Genérico</t>
+          <t>Electrocables</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>TB-KIT-30</t>
+          <t>THHN-8AWG-CU</t>
         </is>
       </c>
       <c r="I21" s="4" t="n">
-        <v>38</v>
+        <v>2.45</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>38</v>
+        <v>130.09</v>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="N21" s="3" t="n">
-        <v>86.5</v>
+        <v>88.7</v>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
@@ -1926,164 +1926,6 @@
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
-        <is>
-          <t>PriceGuard: VERDE (86.5%). Genérico TB-KIT-30, Suministros El Oro, Machala.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>wiring_pack</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Cableado</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Consumibles de cableado de tablero</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Suministros El Oro</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Genérico</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>WP-LOCAL</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="n">
-        <v>98</v>
-      </c>
-      <c r="J22" s="4" t="n">
-        <v>98</v>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>confirmado</t>
-        </is>
-      </c>
-      <c r="L22" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="M22" s="3" t="inlineStr">
-        <is>
-          <t>verde</t>
-        </is>
-      </c>
-      <c r="N22" s="3" t="n">
-        <v>85.8</v>
-      </c>
-      <c r="O22" s="3" t="inlineStr">
-        <is>
-          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
-        </is>
-      </c>
-      <c r="P22" s="3" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="Q22" s="3" t="inlineStr">
-        <is>
-          <t>PriceGuard: VERDE (85.8%). Genérico WP-LOCAL, Suministros El Oro, Machala.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>power_cable</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Cableado</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Conductor de fuerza</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Suministros El Oro</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Electrocables</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>THHN-8AWG-CU</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="J23" s="4" t="n">
-        <v>130.09</v>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>confirmado</t>
-        </is>
-      </c>
-      <c r="L23" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="inlineStr">
-        <is>
-          <t>verde</t>
-        </is>
-      </c>
-      <c r="N23" s="3" t="n">
-        <v>88.7</v>
-      </c>
-      <c r="O23" s="3" t="inlineStr">
-        <is>
-          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
-        </is>
-      </c>
-      <c r="P23" s="3" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>PriceGuard: VERDE (88.7%). Electrocables THHN-8AWG-CU, Suministros El Oro, Machala.</t>
         </is>
@@ -2143,7 +1985,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>19/19</t>
+          <t>17/17</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2007,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>83.0%</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2019,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verde 17 / Amarillo 1 / Rojo 1</t>
+          <t>Verde 15 / Amarillo 1 / Rojo 1</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2030,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2963.59</v>
+        <v>2854.59</v>
       </c>
     </row>
     <row r="8">
@@ -2198,7 +2040,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5742.35</v>
+        <v>5595.2</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Actualizar a ControlPro V13 FitLock Pro
</commit_message>
<xml_diff>
--- a/deliverables/SAMPLE_BOM_PRICEGUARD.xlsx
+++ b/deliverables/SAMPLE_BOM_PRICEGUARD.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -670,7 +670,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>overload_relay</t>
+          <t>contactor_fwd</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Relé de sobrecarga</t>
+          <t>Contactor de línea / seguridad para VFD</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -703,14 +703,14 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>LRD3357</t>
+          <t>LC1D32G7</t>
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="N6" s="3" t="n">
-        <v>88.09999999999999</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
@@ -742,14 +742,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (88.1%). Schneider LRD3357, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (91.4%). Schneider LC1D32G7, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>contactor_fwd</t>
+          <t>vfd</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Contactor de línea / seguridad para VFD</t>
+          <t>Variador de frecuencia</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -772,33 +772,33 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Cuenca Control Supply</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>LC1D32G7</t>
+          <t>ACS580-01-039A-4</t>
         </is>
       </c>
       <c r="I7" s="4" t="n">
-        <v>82</v>
+        <v>1180</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>82</v>
+        <v>1180</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>referencial fuerte</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media-alta</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="N7" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
@@ -821,14 +821,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (91.4%). Schneider LC1D32G7, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (80.7%). ABB ACS580-01-039A-4, Cuenca Control Supply, Cuenca.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>vfd</t>
+          <t>line_reactor</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Variador de frecuencia</t>
+          <t>Reactor de línea</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -851,46 +851,46 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Cuenca Control Supply</t>
+          <t>Suministros El Oro</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Genérico industrial</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>ACS580-01-039A-4</t>
+          <t>LR-25HP-460</t>
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1180</v>
+        <v>168</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1180</v>
+        <v>168</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>referencial fuerte</t>
+          <t>referencial</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>media-alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>verde</t>
+          <t>amarillo</t>
         </is>
       </c>
       <c r="N8" s="3" t="n">
-        <v>80.7</v>
+        <v>75</v>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
+          <t>Usar como referencia; enviar RFQ si el proyecto es sensible a precio o plazo.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -900,14 +900,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (80.7%). ABB ACS580-01-039A-4, Cuenca Control Supply, Cuenca.</t>
+          <t>PriceGuard: AMARILLO (75.0%). Genérico industrial LR-25HP-460, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>line_reactor</t>
+          <t>braking_resistor</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Reactor de línea</t>
+          <t>Resistencia de frenado</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -930,73 +930,73 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Suministros El Oro</t>
+          <t>Automatización Andina</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Genérico industrial</t>
+          <t>Danfoss</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>LR-25HP-460</t>
+          <t>BR-25HP</t>
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>168</v>
+        <v>247.5</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>168</v>
+        <v>247.5</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>referencial</t>
+          <t>estimado corregido</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>baja</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>amarillo</t>
+          <t>rojo</t>
         </is>
       </c>
       <c r="N9" s="3" t="n">
-        <v>75</v>
+        <v>50.8</v>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Usar como referencia; enviar RFQ si el proyecto es sensible a precio o plazo.</t>
+          <t>Precio fuera de confianza. Usar mediana temporal y enviar RFQ a varios proveedores.</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>available</t>
+          <t>quote_needed</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: AMARILLO (75.0%). Genérico industrial LR-25HP-460, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: ROJO (50.8%). Danfoss BR-25HP, Automatización Andina, Quito. Alertas: stock no confirmado. Se aplicó autocorrección por banda de mercado.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>braking_resistor</t>
+          <t>phase_monitor</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Fuerza</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Resistencia de frenado</t>
+          <t>Relé monitor de fase</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -1009,73 +1009,73 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Automatización Andina</t>
+          <t>ElectroIndustrial Guayaquil</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Danfoss</t>
+          <t>Schneider</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>BR-25HP</t>
+          <t>RM22TR33</t>
         </is>
       </c>
       <c r="I10" s="4" t="n">
-        <v>247.5</v>
+        <v>94</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>247.5</v>
+        <v>94</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>estimado corregido</t>
+          <t>confirmado</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>rojo</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="N10" s="3" t="n">
-        <v>50.8</v>
+        <v>86.3</v>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Precio fuera de confianza. Usar mediana temporal y enviar RFQ a varios proveedores.</t>
+          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>quote_needed</t>
+          <t>available</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: ROJO (50.8%). Danfoss BR-25HP, Automatización Andina, Quito. Alertas: stock no confirmado. Se aplicó autocorrección por banda de mercado.</t>
+          <t>PriceGuard: VERDE (86.3%). Schneider RM22TR33, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>phase_monitor</t>
+          <t>control_transformer</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Relé monitor de fase</t>
+          <t>Transformador de control</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -1088,24 +1088,24 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Suministros El Oro</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>Genérico industrial</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>RM22TR33</t>
+          <t>TC-2KVA</t>
         </is>
       </c>
       <c r="I11" s="4" t="n">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
         </is>
       </c>
       <c r="N11" s="3" t="n">
-        <v>86.3</v>
+        <v>86.2</v>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
@@ -1137,24 +1137,24 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.3%). Schneider RM22TR33, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (86.2%). Genérico industrial TC-2KVA, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>control_transformer</t>
+          <t>cabinet</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Tablero</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Transformador de control</t>
+          <t>Gabinete industrial</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -1172,19 +1172,19 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Genérico industrial</t>
+          <t>Metálico Nacional</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>TC-2KVA</t>
+          <t>MN-604025</t>
         </is>
       </c>
       <c r="I12" s="4" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="N12" s="3" t="n">
-        <v>86.2</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
@@ -1216,24 +1216,24 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.2%). Genérico industrial TC-2KVA, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (84.9%). Metálico Nacional MN-604025, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>cabinet</t>
+          <t>estop</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Tablero</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Gabinete industrial</t>
+          <t>Paro de emergencia</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -1246,24 +1246,24 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Suministros El Oro</t>
+          <t>ElectroIndustrial Guayaquil</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Metálico Nacional</t>
+          <t>Schneider</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>MN-604025</t>
+          <t>XB4BS542</t>
         </is>
       </c>
       <c r="I13" s="4" t="n">
-        <v>135</v>
+        <v>24</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>135</v>
+        <v>24</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="N13" s="3" t="n">
-        <v>84.90000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
@@ -1295,24 +1295,24 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (84.9%). Metálico Nacional MN-604025, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (87.2%). Schneider XB4BS542, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>estop</t>
+          <t>pushbuttons</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Paro de emergencia</t>
+          <t>Botonera de mando</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -1335,14 +1335,14 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>XB4BS542</t>
+          <t>XB4 Kit</t>
         </is>
       </c>
       <c r="I14" s="4" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="N14" s="3" t="n">
-        <v>87.2</v>
+        <v>86.5</v>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
@@ -1374,28 +1374,28 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (87.2%). Schneider XB4BS542, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (86.5%). Schneider XB4 Kit, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>pushbuttons</t>
+          <t>limit_switches</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Botonera de mando</t>
+          <t>Finales de carrera</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
@@ -1414,14 +1414,14 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>XB4 Kit</t>
+          <t>XCK-M</t>
         </is>
       </c>
       <c r="I15" s="4" t="n">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="N15" s="3" t="n">
-        <v>86.5</v>
+        <v>86.8</v>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
@@ -1453,28 +1453,28 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.5%). Schneider XB4 Kit, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (86.8%). Schneider XCK-M, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>limit_switches</t>
+          <t>brake_rectifier</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Finales de carrera</t>
+          <t>Control/rectificador de freno</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
@@ -1483,33 +1483,33 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Proveedor Premium Quito</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>Bonfiglioli</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>XCK-M</t>
+          <t>BRE120</t>
         </is>
       </c>
       <c r="I16" s="4" t="n">
-        <v>38</v>
+        <v>142</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>76</v>
+        <v>142</v>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>referencial</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="N16" s="3" t="n">
-        <v>86.8</v>
+        <v>77.7</v>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
@@ -1532,24 +1532,24 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.8%). Schneider XCK-M, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (77.7%). Bonfiglioli BRE120, Proveedor Premium Quito, Quito.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>brake_rectifier</t>
+          <t>label_package</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Taller</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Control/rectificador de freno</t>
+          <t>Etiquetado premium</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -1562,33 +1562,33 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Proveedor Premium Quito</t>
+          <t>Suministros El Oro</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Bonfiglioli</t>
+          <t>Genérico</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>BRE120</t>
+          <t>LABEL-KIT</t>
         </is>
       </c>
       <c r="I17" s="4" t="n">
-        <v>142</v>
+        <v>32</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>142</v>
+        <v>32</v>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>referencial</t>
+          <t>confirmado</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="N17" s="3" t="n">
-        <v>77.7</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
@@ -1611,24 +1611,24 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (77.7%). Bonfiglioli BRE120, Proveedor Premium Quito, Quito.</t>
+          <t>PriceGuard: VERDE (81.1%). Genérico LABEL-KIT, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>label_package</t>
+          <t>terminal_blocks</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Taller</t>
+          <t>Cableado</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Etiquetado premium</t>
+          <t>Borneras, puentes y marcadores</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -1651,14 +1651,14 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>LABEL-KIT</t>
+          <t>TB-KIT-30</t>
         </is>
       </c>
       <c r="I18" s="4" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
         </is>
       </c>
       <c r="N18" s="3" t="n">
-        <v>81.09999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
@@ -1690,14 +1690,14 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (81.1%). Genérico LABEL-KIT, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (86.5%). Genérico TB-KIT-30, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>terminal_blocks</t>
+          <t>wiring_pack</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Borneras, puentes y marcadores</t>
+          <t>Consumibles de cableado de tablero</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -1730,14 +1730,14 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>TB-KIT-30</t>
+          <t>WP-LOCAL</t>
         </is>
       </c>
       <c r="I19" s="4" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="N19" s="3" t="n">
-        <v>86.5</v>
+        <v>85.8</v>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
@@ -1769,14 +1769,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.5%). Genérico TB-KIT-30, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (85.8%). Genérico WP-LOCAL, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>wiring_pack</t>
+          <t>power_cable</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1786,15 +1786,15 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Consumibles de cableado de tablero</t>
+          <t>Conductor de fuerza</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1</v>
+        <v>53.1</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1804,19 +1804,19 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Genérico</t>
+          <t>Electrocables</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>WP-LOCAL</t>
+          <t>THHN-8AWG-CU</t>
         </is>
       </c>
       <c r="I20" s="4" t="n">
-        <v>98</v>
+        <v>2.45</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>98</v>
+        <v>130.09</v>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="N20" s="3" t="n">
-        <v>85.8</v>
+        <v>88.7</v>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
@@ -1847,85 +1847,6 @@
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
-        <is>
-          <t>PriceGuard: VERDE (85.8%). Genérico WP-LOCAL, Suministros El Oro, Machala.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>power_cable</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Cableado</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Conductor de fuerza</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Suministros El Oro</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Electrocables</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>THHN-8AWG-CU</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="J21" s="4" t="n">
-        <v>130.09</v>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>confirmado</t>
-        </is>
-      </c>
-      <c r="L21" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>verde</t>
-        </is>
-      </c>
-      <c r="N21" s="3" t="n">
-        <v>88.7</v>
-      </c>
-      <c r="O21" s="3" t="inlineStr">
-        <is>
-          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
-        </is>
-      </c>
-      <c r="P21" s="3" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="Q21" s="3" t="inlineStr">
         <is>
           <t>PriceGuard: VERDE (88.7%). Electrocables THHN-8AWG-CU, Suministros El Oro, Machala.</t>
         </is>
@@ -1985,7 +1906,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>17/17</t>
+          <t>16/16</t>
         </is>
       </c>
     </row>
@@ -2007,7 +1928,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>83.0%</t>
+          <t>82.7%</t>
         </is>
       </c>
     </row>
@@ -2019,7 +1940,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verde 15 / Amarillo 1 / Rojo 1</t>
+          <t>Verde 14 / Amarillo 1 / Rojo 1</t>
         </is>
       </c>
     </row>
@@ -2030,7 +1951,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2854.59</v>
+        <v>2788.59</v>
       </c>
     </row>
     <row r="8">
@@ -2040,7 +1961,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5595.2</v>
+        <v>5506.1</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Actualizar a ControlPro V15 OptionTrust Pro
</commit_message>
<xml_diff>
--- a/deliverables/SAMPLE_BOM_PRICEGUARD.xlsx
+++ b/deliverables/SAMPLE_BOM_PRICEGUARD.xlsx
@@ -490,14 +490,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ControlPro Advisor OS V12 - BOM cotizable</t>
+          <t>ControlPro Advisor OS V15 - BOM cotizable</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Proyecto: Guinche de izaje — Cotización técnica premium</t>
+          <t>Proyecto: Bomba industrial — Arranque protegido</t>
         </is>
       </c>
     </row>
@@ -624,23 +624,23 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>EasyPact CVS 60A 25kA</t>
+          <t>EasyPact CVS 25A 25kA</t>
         </is>
       </c>
       <c r="I5" s="4" t="n">
-        <v>145</v>
+        <v>88</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>145</v>
+        <v>88</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>referencial</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="N5" s="3" t="n">
-        <v>88</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
@@ -663,14 +663,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (88.0%). Schneider EasyPact CVS 60A 25kA, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (76.1%). Schneider EasyPact CVS 25A 25kA, ElectroIndustrial Guayaquil, Guayaquil. FitLock rechazó ofertas incompatibles: Schneider EasyPact CVS 60A 25kA: FitLock: oferta clase 600 V no corresponde a proyecto 220 V | ABB Tmax XT1 60A: FitLock: oferta clase 600 V no corresponde a proyecto 220 V | Chint NXM-63S 60A: FitLock: oferta clase 600 V no corresponde a proyecto 220 V.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>contactor_fwd</t>
+          <t>overload_relay</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Contactor de línea / seguridad para VFD</t>
+          <t>Relé de sobrecarga</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -703,14 +703,14 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>LC1D32G7</t>
+          <t>LRD3357</t>
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="N6" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>90.7</v>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
@@ -742,14 +742,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (91.4%). Schneider LC1D32G7, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (90.7%). Schneider LRD3357, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>vfd</t>
+          <t>contactor_fwd</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Variador de frecuencia</t>
+          <t>Contactor principal</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -772,33 +772,33 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Cuenca Control Supply</t>
+          <t>ElectroIndustrial Guayaquil</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Schneider</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>ACS580-01-039A-4</t>
+          <t>LC1D32G7</t>
         </is>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1180</v>
+        <v>82</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>1180</v>
+        <v>82</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>referencial fuerte</t>
+          <t>confirmado</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>media-alta</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="N7" s="3" t="n">
-        <v>80.7</v>
+        <v>91.3</v>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
@@ -821,14 +821,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (80.7%). ABB ACS580-01-039A-4, Cuenca Control Supply, Cuenca.</t>
+          <t>PriceGuard: VERDE (91.3%). Schneider LC1D32G7, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>line_reactor</t>
+          <t>soft_starter</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Reactor de línea</t>
+          <t>Soft starter</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -856,41 +856,41 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Genérico industrial</t>
+          <t>Chint</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>LR-25HP-460</t>
+          <t>NJRP2-32-220</t>
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>168</v>
+        <v>285</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>168</v>
+        <v>285</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>referencial</t>
+          <t>referencial fuerte</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>media-alta</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>amarillo</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="N8" s="3" t="n">
-        <v>75</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Usar como referencia; enviar RFQ si el proyecto es sensible a precio o plazo.</t>
+          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -900,14 +900,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: AMARILLO (75.0%). Genérico industrial LR-25HP-460, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (78.4%). Chint NJRP2-32-220, Suministros El Oro, Machala. FitLock rechazó ofertas incompatibles: Schneider ATS22D47S6: FitLock: oferta clase 460 V no corresponde a proyecto 220 V | ABB PSE45: FitLock: oferta sin corriente verificable para requerimiento 14 A; FitLock: oferta clase 460 V no corresponde a proyecto 220 V | Chint NJRP2-45: FitLock: oferta sin corriente verificable para requerimiento 14 A; FitLock: oferta clase 460 V no corresponde a proyecto 220 V.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>braking_resistor</t>
+          <t>bypass_contactor</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Resistencia de frenado</t>
+          <t>Contactor bypass</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -930,56 +930,56 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Automatización Andina</t>
+          <t>ElectroIndustrial Guayaquil</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Danfoss</t>
+          <t>Schneider</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>BR-25HP</t>
+          <t>LC1D50G7</t>
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>247.5</v>
+        <v>118</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>247.5</v>
+        <v>118</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>estimado corregido</t>
+          <t>referencial fuerte</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>media-alta</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>rojo</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="N9" s="3" t="n">
-        <v>50.8</v>
+        <v>79.3</v>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Precio fuera de confianza. Usar mediana temporal y enviar RFQ a varios proveedores.</t>
+          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>quote_needed</t>
+          <t>available</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: ROJO (50.8%). Danfoss BR-25HP, Automatización Andina, Quito. Alertas: stock no confirmado. Se aplicó autocorrección por banda de mercado.</t>
+          <t>PriceGuard: VERDE (79.3%). Schneider LC1D50G7, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
@@ -1381,21 +1381,21 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>limit_switches</t>
+          <t>dry_run_protection</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Instrumentación</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Finales de carrera</t>
+          <t>Protección contra trabajo en seco</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
@@ -1404,33 +1404,33 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Suministros El Oro</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>Finder</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>XCK-M</t>
+          <t>DRY-RUN-KIT</t>
         </is>
       </c>
       <c r="I15" s="4" t="n">
-        <v>38</v>
+        <v>115</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>referencial fuerte</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media-alta</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="N15" s="3" t="n">
-        <v>86.8</v>
+        <v>78</v>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
@@ -1453,24 +1453,24 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (86.8%). Schneider XCK-M, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (78.0%). Finder DRY-RUN-KIT, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>brake_rectifier</t>
+          <t>pressure_sensor</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Instrumentación</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Control/rectificador de freno</t>
+          <t>Sensor/presostato de presión</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -1483,24 +1483,24 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Proveedor Premium Quito</t>
+          <t>Suministros El Oro</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Bonfiglioli</t>
+          <t>Danfoss</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>BRE120</t>
+          <t>KP36</t>
         </is>
       </c>
       <c r="I16" s="4" t="n">
-        <v>142</v>
+        <v>68</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>142</v>
+        <v>68</v>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="N16" s="3" t="n">
-        <v>77.7</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (77.7%). Bonfiglioli BRE120, Proveedor Premium Quito, Quito.</t>
+          <t>PriceGuard: VERDE (77.1%). Danfoss KP36, Suministros El Oro, Machala.</t>
         </is>
       </c>
     </row>
@@ -1809,14 +1809,14 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>THHN-8AWG-CU</t>
+          <t>THHN-12AWG-CU</t>
         </is>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2.45</v>
+        <v>0.95</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>130.09</v>
+        <v>50.45</v>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="N20" s="3" t="n">
-        <v>88.7</v>
+        <v>84.8</v>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (88.7%). Electrocables THHN-8AWG-CU, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (84.8%). Electrocables THHN-12AWG-CU, Suministros El Oro, Machala. FitLock rechazó ofertas incompatibles: Electrocables THHN-10AWG-CU: FitLock: cable ofertado #10 AWG no coincide con cálculo preliminar #12 AWG | Electrocables THHN-8AWG-CU: FitLock: cable ofertado #8 AWG no coincide con cálculo preliminar #12 AWG | Electrocables THHN-6AWG-CU: FitLock: cable ofertado #6 AWG no coincide con cálculo preliminar #12 AWG | Cablec THHN-8AWG: FitLock: cable ofertado #8 AWG no coincide con cálculo preliminar #12 AWG.</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>82.7%</t>
+          <t>83.8%</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verde 14 / Amarillo 1 / Rojo 1</t>
+          <t>Verde 16 / Amarillo 0 / Rojo 0</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2788.59</v>
+        <v>1490.45</v>
       </c>
     </row>
     <row r="8">
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5506.1</v>
+        <v>3591.61</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Actualizar a ControlPro V16 MarketVision Pro
</commit_message>
<xml_diff>
--- a/deliverables/SAMPLE_BOM_PRICEGUARD.xlsx
+++ b/deliverables/SAMPLE_BOM_PRICEGUARD.xlsx
@@ -490,14 +490,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ControlPro Advisor OS V15 - BOM cotizable</t>
+          <t>ControlPro Advisor OS V16 - BOM cotizable</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Proyecto: Bomba industrial — Arranque protegido</t>
+          <t>Proyecto: Guinche de izaje — Cotización técnica premium</t>
         </is>
       </c>
     </row>
@@ -624,33 +624,33 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>EasyPact CVS 25A 25kA</t>
+          <t>EasyPact CVS 60A 25kA</t>
         </is>
       </c>
       <c r="I5" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="n">
         <v>88</v>
       </c>
-      <c r="J5" s="4" t="n">
-        <v>88</v>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>referencial</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>verde</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="n">
-        <v>76.09999999999999</v>
-      </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
           <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
@@ -663,14 +663,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (76.1%). Schneider EasyPact CVS 25A 25kA, ElectroIndustrial Guayaquil, Guayaquil. FitLock rechazó ofertas incompatibles: Schneider EasyPact CVS 60A 25kA: FitLock: oferta clase 600 V no corresponde a proyecto 220 V | ABB Tmax XT1 60A: FitLock: oferta clase 600 V no corresponde a proyecto 220 V | Chint NXM-63S 60A: FitLock: oferta clase 600 V no corresponde a proyecto 220 V.</t>
+          <t>PriceGuard: VERDE (88.0%). Schneider EasyPact CVS 60A 25kA, ElectroIndustrial Guayaquil, Guayaquil. FitLock rechazó ofertas incompatibles: Schneider EasyPact CVS 25A 25kA: FitLock: corriente ofertada 25 A menor que requerida 60 A; FitLock: oferta clase 240 V menor que proyecto 460 V.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>overload_relay</t>
+          <t>contactor_fwd</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Relé de sobrecarga</t>
+          <t>Contactor de línea / seguridad para VFD</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -703,14 +703,14 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>LRD3357</t>
+          <t>LC1D32G7</t>
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="N6" s="3" t="n">
-        <v>90.7</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
@@ -742,14 +742,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (90.7%). Schneider LRD3357, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (90.4%). Schneider LC1D32G7, ElectroIndustrial Guayaquil, Guayaquil. FitLock rechazó ofertas incompatibles: Schneider LC1D18G7: FitLock: corriente ofertada 18 A menor que requerida 30.4 A | Chint NC1-3210 120V: FitLock: oferta clase 120 V menor que proyecto 460 V.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>contactor_fwd</t>
+          <t>vfd</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Contactor principal</t>
+          <t>Variador de frecuencia</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -772,33 +772,33 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Cuenca Control Supply</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>LC1D32G7</t>
+          <t>ACS580-01-039A-4</t>
         </is>
       </c>
       <c r="I7" s="4" t="n">
-        <v>82</v>
+        <v>1180</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>82</v>
+        <v>1180</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>confirmado</t>
+          <t>referencial fuerte</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media-alta</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="N7" s="3" t="n">
-        <v>91.3</v>
+        <v>80.7</v>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
@@ -821,14 +821,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (91.3%). Schneider LC1D32G7, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: VERDE (80.7%). ABB ACS580-01-039A-4, Cuenca Control Supply, Cuenca. FitLock rechazó ofertas incompatibles: INVT GD200A-7R5G-2: FitLock: oferta 10 HP menor que motor 25 HP; FitLock: oferta clase 220 V menor que proyecto 460 V | Schneider ATV320U75M3C: FitLock: oferta 10 HP menor que motor 25 HP; FitLock: oferta clase 220 V menor que proyecto 460 V.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>soft_starter</t>
+          <t>line_reactor</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Soft starter</t>
+          <t>Reactor de línea</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -856,41 +856,41 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Chint</t>
+          <t>Genérico industrial</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>NJRP2-32-220</t>
+          <t>LR-25HP-460</t>
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>285</v>
+        <v>168</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>285</v>
+        <v>168</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>referencial fuerte</t>
+          <t>referencial</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>media-alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>verde</t>
+          <t>amarillo</t>
         </is>
       </c>
       <c r="N8" s="3" t="n">
-        <v>78.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
+          <t>Usar como referencia; enviar RFQ si el proyecto es sensible a precio o plazo.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -900,14 +900,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (78.4%). Chint NJRP2-32-220, Suministros El Oro, Machala. FitLock rechazó ofertas incompatibles: Schneider ATS22D47S6: FitLock: oferta clase 460 V no corresponde a proyecto 220 V | ABB PSE45: FitLock: oferta sin corriente verificable para requerimiento 14 A; FitLock: oferta clase 460 V no corresponde a proyecto 220 V | Chint NJRP2-45: FitLock: oferta sin corriente verificable para requerimiento 14 A; FitLock: oferta clase 460 V no corresponde a proyecto 220 V.</t>
+          <t>PriceGuard: AMARILLO (75.0%). Genérico industrial LR-25HP-460, Suministros El Oro, Machala. FitLock rechazó ofertas incompatibles: Genérico industrial LR-10HP-220: FitLock: oferta 10 HP menor que motor 25 HP; FitLock: oferta clase 220 V menor que proyecto 460 V | MTE RL-010HP-220: FitLock: oferta 10 HP menor que motor 25 HP; FitLock: oferta clase 220 V menor que proyecto 460 V.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>bypass_contactor</t>
+          <t>braking_resistor</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Contactor bypass</t>
+          <t>Resistencia de frenado</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -930,56 +930,56 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>ElectroIndustrial Guayaquil</t>
+          <t>Automatización Andina</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Schneider</t>
+          <t>Danfoss</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>LC1D50G7</t>
+          <t>BR-25HP</t>
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>118</v>
+        <v>247.5</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>118</v>
+        <v>247.5</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>referencial fuerte</t>
+          <t>estimado corregido</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>media-alta</t>
+          <t>baja</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>verde</t>
+          <t>rojo</t>
         </is>
       </c>
       <c r="N9" s="3" t="n">
-        <v>79.3</v>
+        <v>50.8</v>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Usar en cotización revisable; confirmar vigencia si la oferta supera 72 horas.</t>
+          <t>Precio fuera de confianza. Usar mediana temporal y enviar RFQ a varios proveedores.</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>available</t>
+          <t>quote_needed</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (79.3%). Schneider LC1D50G7, ElectroIndustrial Guayaquil, Guayaquil.</t>
+          <t>PriceGuard: ROJO (50.8%). Danfoss BR-25HP, Automatización Andina, Quito. Alertas: stock no confirmado. Se aplicó autocorrección por banda de mercado.</t>
         </is>
       </c>
     </row>
@@ -1381,21 +1381,21 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>dry_run_protection</t>
+          <t>limit_switches</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Instrumentación</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Protección contra trabajo en seco</t>
+          <t>Finales de carrera</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
@@ -1404,33 +1404,33 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Suministros El Oro</t>
+          <t>ElectroIndustrial Guayaquil</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Finder</t>
+          <t>Schneider</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>DRY-RUN-KIT</t>
+          <t>XCK-M</t>
         </is>
       </c>
       <c r="I15" s="4" t="n">
-        <v>115</v>
+        <v>38</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>referencial fuerte</t>
+          <t>confirmado</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>media-alta</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="N15" s="3" t="n">
-        <v>78</v>
+        <v>86.8</v>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
@@ -1453,24 +1453,24 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (78.0%). Finder DRY-RUN-KIT, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (86.8%). Schneider XCK-M, ElectroIndustrial Guayaquil, Guayaquil.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>pressure_sensor</t>
+          <t>brake_rectifier</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Instrumentación</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Sensor/presostato de presión</t>
+          <t>Control/rectificador de freno</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -1483,24 +1483,24 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Suministros El Oro</t>
+          <t>Proveedor Premium Quito</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Danfoss</t>
+          <t>Bonfiglioli</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>KP36</t>
+          <t>BRE120</t>
         </is>
       </c>
       <c r="I16" s="4" t="n">
-        <v>68</v>
+        <v>142</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>68</v>
+        <v>142</v>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="N16" s="3" t="n">
-        <v>77.09999999999999</v>
+        <v>77.7</v>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (77.1%). Danfoss KP36, Suministros El Oro, Machala.</t>
+          <t>PriceGuard: VERDE (77.7%). Bonfiglioli BRE120, Proveedor Premium Quito, Quito.</t>
         </is>
       </c>
     </row>
@@ -1809,14 +1809,14 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>THHN-12AWG-CU</t>
+          <t>THHN-8AWG-CU</t>
         </is>
       </c>
       <c r="I20" s="4" t="n">
-        <v>0.95</v>
+        <v>2.45</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>50.45</v>
+        <v>130.09</v>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="N20" s="3" t="n">
-        <v>84.8</v>
+        <v>88.7</v>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>PriceGuard: VERDE (84.8%). Electrocables THHN-12AWG-CU, Suministros El Oro, Machala. FitLock rechazó ofertas incompatibles: Electrocables THHN-10AWG-CU: FitLock: cable ofertado #10 AWG no coincide con cálculo preliminar #12 AWG | Electrocables THHN-8AWG-CU: FitLock: cable ofertado #8 AWG no coincide con cálculo preliminar #12 AWG | Electrocables THHN-6AWG-CU: FitLock: cable ofertado #6 AWG no coincide con cálculo preliminar #12 AWG | Cablec THHN-8AWG: FitLock: cable ofertado #8 AWG no coincide con cálculo preliminar #12 AWG.</t>
+          <t>PriceGuard: VERDE (88.7%). Electrocables THHN-8AWG-CU, Suministros El Oro, Machala. FitLock rechazó ofertas incompatibles: Electrocables THHN-10AWG-CU: FitLock: cable ofertado #10 AWG no coincide con cálculo preliminar #8 AWG | Electrocables THHN-6AWG-CU: FitLock: cable ofertado #6 AWG no coincide con cálculo preliminar #8 AWG | Electrocables THHN-12AWG-CU: FitLock: cable ofertado #12 AWG no coincide con cálculo preliminar #8 AWG | Electrocables THHN-4AWG-CU: FitLock: cable ofertado #4 AWG no coincide con cálculo preliminar #8 AWG.</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>82.7%</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verde 16 / Amarillo 0 / Rojo 0</t>
+          <t>Verde 14 / Amarillo 1 / Rojo 1</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1490.45</v>
+        <v>2788.59</v>
       </c>
     </row>
     <row r="8">
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3591.61</v>
+        <v>5506.1</v>
       </c>
     </row>
     <row r="9">

</xml_diff>